<commit_message>
Removed Contact Page and Updated Daytrip Options Spreadsheet
</commit_message>
<xml_diff>
--- a/Backend/Static/DaytripOptions.xlsx
+++ b/Backend/Static/DaytripOptions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://roehamptonprod-my.sharepoint.com/personal/fitzmaua_roehampton_ac_uk/Documents/Documents/Year 3/Final Year Project/Website/Backend/Static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{05AF55C7-B2C8-4E84-8BC2-57FDE6D52A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{03F4AF90-9DCF-4204-A122-33260A9DB91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3330" yWindow="3330" windowWidth="21600" windowHeight="11385" xr2:uid="{120C82BE-9163-485E-96E9-EEFED2CE9E6B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{120C82BE-9163-485E-96E9-EEFED2CE9E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="DaytripOptions" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="212" uniqueCount="138">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="212" uniqueCount="141">
   <si>
     <t>Activity Name</t>
   </si>
@@ -131,18 +131,12 @@
     <t>Support Group for Carers of Adults who are Neurodivergent</t>
   </si>
   <si>
-    <t>Kingston Carers Network, Tolworth</t>
-  </si>
-  <si>
     <t>Free (Booking Required)</t>
   </si>
   <si>
     <t>Support Groups</t>
   </si>
   <si>
-    <t>https://www.kingstoncarers.org.uk/calendar/item/52508958</t>
-  </si>
-  <si>
     <t xml:space="preserve">Location </t>
   </si>
   <si>
@@ -230,18 +224,9 @@
     <t>Support Group for Carers of People with a Mental Health Condition</t>
   </si>
   <si>
-    <t>KT6 7HF</t>
-  </si>
-  <si>
     <t>1hr 15mins</t>
   </si>
   <si>
-    <t>https://www.kingstoncarers.org.uk/calendar/item/45438241</t>
-  </si>
-  <si>
-    <t>https://www.kingstoncarers.org.uk/calendar/item/52508959</t>
-  </si>
-  <si>
     <t>London Transport Museum</t>
   </si>
   <si>
@@ -440,19 +425,43 @@
     <t>price_numeric</t>
   </si>
   <si>
-    <t>2026-03-30</t>
-  </si>
-  <si>
-    <t>2026-04-14</t>
-  </si>
-  <si>
-    <t>2026-04-27</t>
-  </si>
-  <si>
     <t>2026-05-12</t>
   </si>
   <si>
     <t>2026-05-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free </t>
+  </si>
+  <si>
+    <t>KT6 6RH</t>
+  </si>
+  <si>
+    <t>Fircroft Trust, 96 Ditton Road</t>
+  </si>
+  <si>
+    <t>Guildhall Building, Kingston Upon Thames</t>
+  </si>
+  <si>
+    <t>KT1 1EU</t>
+  </si>
+  <si>
+    <t>2026-06-09</t>
+  </si>
+  <si>
+    <t>https://www.kingstoncarers.org.uk/calendar/item/45438243</t>
+  </si>
+  <si>
+    <t>2026-06-29</t>
+  </si>
+  <si>
+    <t>https://www.kingstoncarers.org.uk/calendar/item/52508961</t>
+  </si>
+  <si>
+    <t>2026-07-14</t>
+  </si>
+  <si>
+    <t>https://www.kingstoncarers.org.uk/calendar/item/45438244</t>
   </si>
 </sst>
 </file>
@@ -893,37 +902,37 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>2</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>5</v>
@@ -931,7 +940,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -940,7 +949,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>
@@ -955,13 +964,13 @@
         <v>8</v>
       </c>
       <c r="I2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J2">
         <v>210</v>
       </c>
       <c r="K2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>6</v>
@@ -969,7 +978,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -978,7 +987,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s">
         <v>11</v>
@@ -993,13 +1002,13 @@
         <v>8</v>
       </c>
       <c r="I3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J3">
         <v>1440</v>
       </c>
       <c r="K3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L3" s="1" t="s">
         <v>28</v>
@@ -1007,7 +1016,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
@@ -1016,7 +1025,7 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
         <v>20</v>
@@ -1031,13 +1040,13 @@
         <v>8</v>
       </c>
       <c r="I4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J4">
         <v>240</v>
       </c>
       <c r="K4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>19</v>
@@ -1045,16 +1054,16 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
@@ -1069,30 +1078,30 @@
         <v>8</v>
       </c>
       <c r="I5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J5">
         <v>150</v>
       </c>
       <c r="K5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E6" t="s">
         <v>11</v>
@@ -1107,21 +1116,21 @@
         <v>8</v>
       </c>
       <c r="I6" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="J6">
         <v>120</v>
       </c>
       <c r="K6" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -1130,7 +1139,7 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E7" t="s">
         <v>22</v>
@@ -1145,13 +1154,13 @@
         <v>8</v>
       </c>
       <c r="I7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J7">
         <v>150</v>
       </c>
       <c r="K7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>21</v>
@@ -1159,16 +1168,16 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" t="s">
         <v>39</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" t="s">
-        <v>41</v>
       </c>
       <c r="E8" t="s">
         <v>22</v>
@@ -1183,30 +1192,30 @@
         <v>8</v>
       </c>
       <c r="I8" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="J8">
         <v>120</v>
       </c>
       <c r="K8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D9" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
@@ -1221,30 +1230,30 @@
         <v>8</v>
       </c>
       <c r="I9" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="J9">
         <v>180</v>
       </c>
       <c r="K9" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D10" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E10" t="s">
         <v>22</v>
@@ -1259,30 +1268,30 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="J10">
         <v>180</v>
       </c>
       <c r="K10" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D11" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E11" t="s">
         <v>22</v>
@@ -1297,21 +1306,21 @@
         <v>8</v>
       </c>
       <c r="I11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J11">
         <v>150</v>
       </c>
       <c r="K11" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B12" t="s">
         <v>17</v>
@@ -1320,7 +1329,7 @@
         <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
         <v>23</v>
@@ -1335,13 +1344,13 @@
         <v>8</v>
       </c>
       <c r="I12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J12">
         <v>198</v>
       </c>
       <c r="K12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>25</v>
@@ -1349,7 +1358,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
@@ -1358,7 +1367,7 @@
         <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
         <v>23</v>
@@ -1373,13 +1382,13 @@
         <v>8</v>
       </c>
       <c r="I13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J13">
         <v>150</v>
       </c>
       <c r="K13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L13" s="1" t="s">
         <v>27</v>
@@ -1387,19 +1396,19 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" t="s">
         <v>73</v>
-      </c>
-      <c r="C14" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E14" t="s">
-        <v>78</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -1411,33 +1420,33 @@
         <v>8</v>
       </c>
       <c r="I14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="J14">
         <v>270</v>
       </c>
       <c r="K14" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E15" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1449,30 +1458,30 @@
         <v>8</v>
       </c>
       <c r="I15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J15">
         <v>150</v>
       </c>
       <c r="K15" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C16" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D16" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E16" t="s">
         <v>11</v>
@@ -1487,206 +1496,206 @@
         <v>8</v>
       </c>
       <c r="I16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J16">
         <v>150</v>
       </c>
       <c r="K16" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" t="s">
+        <v>132</v>
+      </c>
+      <c r="D17" t="s">
         <v>131</v>
       </c>
-      <c r="B17" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" t="s">
-        <v>63</v>
-      </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>130</v>
       </c>
       <c r="F17">
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J17">
-        <v>120</v>
+        <v>75</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B18" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" t="s">
+        <v>134</v>
+      </c>
+      <c r="E18" t="s">
         <v>30</v>
-      </c>
-      <c r="D18" t="s">
-        <v>63</v>
-      </c>
-      <c r="E18" t="s">
-        <v>11</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="I18" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="J18">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" t="s">
+        <v>132</v>
+      </c>
+      <c r="D19" t="s">
         <v>131</v>
       </c>
-      <c r="B19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" t="s">
-        <v>63</v>
-      </c>
       <c r="E19" t="s">
-        <v>31</v>
+        <v>130</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H19" s="8" t="s">
         <v>135</v>
       </c>
       <c r="I19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J19">
-        <v>120</v>
+        <v>75</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>66</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="C20" t="s">
+        <v>133</v>
+      </c>
+      <c r="D20" t="s">
+        <v>134</v>
+      </c>
+      <c r="E20" t="s">
         <v>30</v>
-      </c>
-      <c r="D20" t="s">
-        <v>63</v>
-      </c>
-      <c r="E20" t="s">
-        <v>11</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I20" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="J20">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>96</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>126</v>
+      </c>
+      <c r="B21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" t="s">
         <v>131</v>
       </c>
-      <c r="B21" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" t="s">
-        <v>63</v>
-      </c>
       <c r="E21" t="s">
-        <v>31</v>
+        <v>130</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J21">
-        <v>120</v>
+        <v>75</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1697,16 +1706,15 @@
     <hyperlink ref="L12" r:id="rId4" xr:uid="{C4CBCDA1-B05F-42BA-898F-5ABC4F5F64DC}"/>
     <hyperlink ref="L13" r:id="rId5" xr:uid="{79CD891E-3076-45E3-A3BF-9889368E372F}"/>
     <hyperlink ref="L3" r:id="rId6" xr:uid="{D2C6E130-915D-4A83-971B-2E8E3F24275F}"/>
-    <hyperlink ref="L17" r:id="rId7" xr:uid="{B43F315C-D384-487B-885D-A367BB4EBD80}"/>
-    <hyperlink ref="L18" r:id="rId8" xr:uid="{41B602E5-31E1-47A4-8C7F-BADE841350F4}"/>
-    <hyperlink ref="L19" r:id="rId9" xr:uid="{3EA71444-A2A0-4928-BC10-4D804F791DEE}"/>
-    <hyperlink ref="L15" r:id="rId10" xr:uid="{D8DB663E-F3B4-423A-8D83-323F7E698E74}"/>
-    <hyperlink ref="L5" r:id="rId11" xr:uid="{5715AFC7-D8B8-4D8F-894C-FD49F442CC42}"/>
-    <hyperlink ref="L10" r:id="rId12" xr:uid="{067C58E1-0D1B-4B50-81AD-7F73A292648B}"/>
-    <hyperlink ref="L20" r:id="rId13" xr:uid="{AE8E4A13-CCBE-4408-B494-E5B83A3AA92B}"/>
-    <hyperlink ref="L21" r:id="rId14" xr:uid="{38FC86D6-8630-4198-BE30-949636B49104}"/>
+    <hyperlink ref="L19" r:id="rId7" xr:uid="{3EA71444-A2A0-4928-BC10-4D804F791DEE}"/>
+    <hyperlink ref="L15" r:id="rId8" xr:uid="{D8DB663E-F3B4-423A-8D83-323F7E698E74}"/>
+    <hyperlink ref="L5" r:id="rId9" xr:uid="{5715AFC7-D8B8-4D8F-894C-FD49F442CC42}"/>
+    <hyperlink ref="L10" r:id="rId10" xr:uid="{067C58E1-0D1B-4B50-81AD-7F73A292648B}"/>
+    <hyperlink ref="L20" r:id="rId11" xr:uid="{AE8E4A13-CCBE-4408-B494-E5B83A3AA92B}"/>
+    <hyperlink ref="L21" r:id="rId12" xr:uid="{38FC86D6-8630-4198-BE30-949636B49104}"/>
+    <hyperlink ref="L17" r:id="rId13" xr:uid="{9C5242EF-579E-4B2C-9E54-36A388884E6C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Daytrip Options Spreadsheet
</commit_message>
<xml_diff>
--- a/Backend/Static/DaytripOptions.xlsx
+++ b/Backend/Static/DaytripOptions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://roehamptonprod-my.sharepoint.com/personal/fitzmaua_roehampton_ac_uk/Documents/Documents/Year 3/Final Year Project/Website/Backend/Static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{03F4AF90-9DCF-4204-A122-33260A9DB91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{B4B68D48-C7BB-40E9-B8EF-E0BB5662FF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{120C82BE-9163-485E-96E9-EEFED2CE9E6B}"/>
   </bookViews>
@@ -200,9 +200,6 @@
     <t>2-3hrs</t>
   </si>
   <si>
-    <t>Varies, typically 10am–6pm</t>
-  </si>
-  <si>
     <t>SW7 5BD</t>
   </si>
   <si>
@@ -254,9 +251,6 @@
     <t>WC1B 3DG</t>
   </si>
   <si>
-    <t>10 am–5 pm most days, except on Fridays where 10am-8:30pm</t>
-  </si>
-  <si>
     <t>https://www.britishmuseum.org/</t>
   </si>
   <si>
@@ -275,9 +269,6 @@
     <t>W2 3LH</t>
   </si>
   <si>
-    <t>6 am–9:45 pm</t>
-  </si>
-  <si>
     <t>https://www.royalparks.org.uk/visit/parks/kensington-gardens</t>
   </si>
   <si>
@@ -462,6 +453,15 @@
   </si>
   <si>
     <t>https://www.kingstoncarers.org.uk/calendar/item/45438244</t>
+  </si>
+  <si>
+    <t>6am–9:45 pm</t>
+  </si>
+  <si>
+    <t>Varies, typically 10am-6pm</t>
+  </si>
+  <si>
+    <t>10am–5 pm most days, except on Fridays where 10am-8:30pm</t>
   </si>
 </sst>
 </file>
@@ -902,7 +902,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>0</v>
@@ -917,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>2</v>
@@ -929,7 +929,7 @@
         <v>36</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="K1" s="7" t="s">
         <v>34</v>
@@ -940,7 +940,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -978,7 +978,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -1016,7 +1016,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
@@ -1054,16 +1054,16 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" t="s">
         <v>75</v>
-      </c>
-      <c r="C5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5" t="s">
-        <v>77</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
@@ -1084,24 +1084,24 @@
         <v>150</v>
       </c>
       <c r="K5" t="s">
-        <v>78</v>
+        <v>138</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D6" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
         <v>11</v>
@@ -1116,21 +1116,21 @@
         <v>8</v>
       </c>
       <c r="I6" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="J6">
         <v>120</v>
       </c>
       <c r="K6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -1160,7 +1160,7 @@
         <v>150</v>
       </c>
       <c r="K7" t="s">
-        <v>53</v>
+        <v>139</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>21</v>
@@ -1168,7 +1168,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
         <v>37</v>
@@ -1192,7 +1192,7 @@
         <v>8</v>
       </c>
       <c r="I8" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="J8">
         <v>120</v>
@@ -1206,16 +1206,16 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
@@ -1230,30 +1230,30 @@
         <v>8</v>
       </c>
       <c r="I9" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J9">
         <v>180</v>
       </c>
       <c r="K9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C10" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E10" t="s">
         <v>22</v>
@@ -1268,30 +1268,30 @@
         <v>8</v>
       </c>
       <c r="I10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J10">
         <v>180</v>
       </c>
       <c r="K10" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B11" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E11" t="s">
         <v>22</v>
@@ -1312,15 +1312,15 @@
         <v>150</v>
       </c>
       <c r="K11" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s">
         <v>17</v>
@@ -1329,7 +1329,7 @@
         <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E12" t="s">
         <v>23</v>
@@ -1350,7 +1350,7 @@
         <v>198</v>
       </c>
       <c r="K12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>25</v>
@@ -1358,7 +1358,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
@@ -1367,7 +1367,7 @@
         <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
         <v>23</v>
@@ -1388,7 +1388,7 @@
         <v>150</v>
       </c>
       <c r="K13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L13" s="1" t="s">
         <v>27</v>
@@ -1396,19 +1396,19 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" t="s">
         <v>68</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>69</v>
       </c>
-      <c r="D14" t="s">
-        <v>70</v>
-      </c>
       <c r="E14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -1420,33 +1420,33 @@
         <v>8</v>
       </c>
       <c r="I14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J14">
         <v>270</v>
       </c>
       <c r="K14" t="s">
-        <v>71</v>
+        <v>140</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" t="s">
         <v>62</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>63</v>
       </c>
-      <c r="D15" t="s">
-        <v>64</v>
-      </c>
       <c r="E15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1464,24 +1464,24 @@
         <v>150</v>
       </c>
       <c r="K15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" t="s">
+        <v>102</v>
+      </c>
+      <c r="D16" t="s">
         <v>104</v>
-      </c>
-      <c r="C16" t="s">
-        <v>105</v>
-      </c>
-      <c r="D16" t="s">
-        <v>107</v>
       </c>
       <c r="E16" t="s">
         <v>11</v>
@@ -1502,27 +1502,27 @@
         <v>150</v>
       </c>
       <c r="K16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C17" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D17" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E17" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1531,33 +1531,33 @@
         <v>31</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J17">
         <v>75</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B18" t="s">
         <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D18" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E18" t="s">
         <v>30</v>
@@ -1569,36 +1569,36 @@
         <v>31</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J18">
         <v>120</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D19" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E19" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1607,33 +1607,33 @@
         <v>31</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="I19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J19">
         <v>75</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B20" t="s">
         <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D20" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E20" t="s">
         <v>30</v>
@@ -1645,36 +1645,36 @@
         <v>31</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="I20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J20">
         <v>120</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C21" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D21" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1683,19 +1683,19 @@
         <v>31</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="I21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J21">
         <v>75</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed spreadsheet issue and commented CSS
</commit_message>
<xml_diff>
--- a/Backend/Static/DaytripOptions.xlsx
+++ b/Backend/Static/DaytripOptions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://roehamptonprod-my.sharepoint.com/personal/fitzmaua_roehampton_ac_uk/Documents/Documents/Year 3/Final Year Project/Website/Backend/Static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{B4B68D48-C7BB-40E9-B8EF-E0BB5662FF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{91D2A3E6-C1DC-412C-9A9B-0771A35CAF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{120C82BE-9163-485E-96E9-EEFED2CE9E6B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="212" uniqueCount="141">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="212" uniqueCount="140">
   <si>
     <t>Activity Name</t>
   </si>
@@ -420,9 +420,6 @@
   </si>
   <si>
     <t>2026-05-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free </t>
   </si>
   <si>
     <t>KT6 6RH</t>
@@ -1084,7 +1081,7 @@
         <v>150</v>
       </c>
       <c r="K5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>76</v>
@@ -1160,7 +1157,7 @@
         <v>150</v>
       </c>
       <c r="K7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>21</v>
@@ -1426,7 +1423,7 @@
         <v>270</v>
       </c>
       <c r="K14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="L14" s="1" t="s">
         <v>70</v>
@@ -1516,13 +1513,13 @@
         <v>59</v>
       </c>
       <c r="C17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D17" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E17" t="s">
-        <v>127</v>
+        <v>11</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1554,10 +1551,10 @@
         <v>29</v>
       </c>
       <c r="C18" t="s">
+        <v>129</v>
+      </c>
+      <c r="D18" t="s">
         <v>130</v>
-      </c>
-      <c r="D18" t="s">
-        <v>131</v>
       </c>
       <c r="E18" t="s">
         <v>30</v>
@@ -1592,13 +1589,13 @@
         <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E19" t="s">
-        <v>127</v>
+        <v>11</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1607,7 +1604,7 @@
         <v>31</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I19" t="s">
         <v>60</v>
@@ -1619,7 +1616,7 @@
         <v>58</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -1630,10 +1627,10 @@
         <v>29</v>
       </c>
       <c r="C20" t="s">
+        <v>129</v>
+      </c>
+      <c r="D20" t="s">
         <v>130</v>
-      </c>
-      <c r="D20" t="s">
-        <v>131</v>
       </c>
       <c r="E20" t="s">
         <v>30</v>
@@ -1645,7 +1642,7 @@
         <v>31</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I20" t="s">
         <v>57</v>
@@ -1657,7 +1654,7 @@
         <v>58</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -1668,13 +1665,13 @@
         <v>59</v>
       </c>
       <c r="C21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E21" t="s">
-        <v>127</v>
+        <v>11</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1683,7 +1680,7 @@
         <v>31</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I21" t="s">
         <v>60</v>
@@ -1695,7 +1692,7 @@
         <v>58</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>